<commit_message>
Fixed timezone and added roll number.
</commit_message>
<xml_diff>
--- a/data/attendance.xlsx
+++ b/data/attendance.xlsx
@@ -36,7 +36,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,12 +53,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EBF3FC"/>
         <bgColor rgb="00EBF3FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,15 +73,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -455,32 +446,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Roll Number</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -489,64 +486,25 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>5023119</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>JADHAV ADITYA SUJIT</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>18:23:52</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>SAWANT AKSHAT SANTOSH</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>18:46:20</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>KHAN ARSALAN AHMED</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>18:46:20</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+          <t>06:09:41</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Present</t>
         </is>

</xml_diff>